<commit_message>
V15 --> Cambiando algun parametro de configuración de la red y para entrenar, añdiendo que los videos malos si introduzcan más veces
</commit_message>
<xml_diff>
--- a/backend/reportes/Datos Ejemplo.xlsx
+++ b/backend/reportes/Datos Ejemplo.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\TFG\backend\reportes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22E9448F-F7E6-4235-8B65-AC4AFC64E5A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C76BA58F-1DEB-40A0-B201-77E0CD78C675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4A3FB1CC-E9D2-41A8-8373-7EE8A5446979}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -532,7 +531,7 @@
         <v>9.5</v>
       </c>
       <c r="G2" s="5">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:159" x14ac:dyDescent="0.3">
@@ -574,7 +573,7 @@
         <v>10</v>
       </c>
       <c r="G4" s="6">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:159" x14ac:dyDescent="0.3">

</xml_diff>